<commit_message>
test: actualiza resultados QA y corrige guardado FAQ
</commit_message>
<xml_diff>
--- a/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
+++ b/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
@@ -4707,7 +4707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -4750,7 +4750,7 @@
         </is>
       </c>
       <c r="E3" s="122" t="n">
-        <v>22</v>
+        <v>59</v>
       </c>
       <c r="G3" s="120" t="inlineStr">
         <is>
@@ -4763,7 +4763,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="123" t="inlineStr">
         <is>
@@ -5840,6 +5839,1745 @@
         </is>
       </c>
       <c r="I27" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="78" customHeight="1">
+      <c r="A28" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B28" s="124" t="inlineStr">
+        <is>
+          <t>MOB-003</t>
+        </is>
+      </c>
+      <c r="C28" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D28" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture con seis lotes e imágenes para validar carrusel y lightbox móvil.</t>
+        </is>
+      </c>
+      <c r="E28" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F28" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA publicado con al menos seis lotes y fotografías, y mantenerlo aislado de los datos generales.</t>
+        </is>
+      </c>
+      <c r="G28" s="124" t="inlineStr">
+        <is>
+          <t>A 375×812 se muestra una tarjeta por vez; ambas flechas y el lightbox funcionan sin desborde.</t>
+        </is>
+      </c>
+      <c r="H28" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I28" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="78" customHeight="1">
+      <c r="A29" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B29" s="124" t="inlineStr">
+        <is>
+          <t>MOB-004</t>
+        </is>
+      </c>
+      <c r="C29" s="125" t="inlineStr">
+        <is>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="D29" s="124" t="inlineStr">
+        <is>
+          <t>La navegación del panel a 390 px no cambia de Resumen a Remates.</t>
+        </is>
+      </c>
+      <c r="E29" s="129" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F29" s="124" t="inlineStr">
+        <is>
+          <t>Revisar el handler de navegación móvil, el cierre del sidebar y posibles capas superpuestas; asegurar que cada botón actualice la sección activa.</t>
+        </is>
+      </c>
+      <c r="G29" s="124" t="inlineStr">
+        <is>
+          <t>A 390×844 se puede recorrer Resumen, Remates y editor sin controles inaccesibles.</t>
+        </is>
+      </c>
+      <c r="H29" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I29" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="78" customHeight="1">
+      <c r="A30" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B30" s="124" t="inlineStr">
+        <is>
+          <t>ACC-A11Y-003</t>
+        </is>
+      </c>
+      <c r="C30" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D30" s="124" t="inlineStr">
+        <is>
+          <t>La automatización no puede aplicar zoom real de navegador al 200%.</t>
+        </is>
+      </c>
+      <c r="E30" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F30" s="124" t="inlineStr">
+        <is>
+          <t>Añadir una prueba E2E/CDP o un protocolo manual reproducible que fije zoom 200%.</t>
+        </is>
+      </c>
+      <c r="G30" s="124" t="inlineStr">
+        <is>
+          <t>Home, detalle y formulario hacen reflow y siguen utilizables a 200%.</t>
+        </is>
+      </c>
+      <c r="H30" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I30" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="78" customHeight="1">
+      <c r="A31" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B31" s="124" t="inlineStr">
+        <is>
+          <t>ACC-A11Y-004</t>
+        </is>
+      </c>
+      <c r="C31" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D31" s="124" t="inlineStr">
+        <is>
+          <t>No se puede emular prefers-reduced-motion desde la automatización actual.</t>
+        </is>
+      </c>
+      <c r="E31" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F31" s="124" t="inlineStr">
+        <is>
+          <t>Incorporar una prueba E2E que emule reduced motion o una comprobación manual en DevTools.</t>
+        </is>
+      </c>
+      <c r="G31" s="124" t="inlineStr">
+        <is>
+          <t>Con reduce activado, las animaciones y desplazamientos se reducen o desactivan.</t>
+        </is>
+      </c>
+      <c r="H31" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I31" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="78" customHeight="1">
+      <c r="A32" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B32" s="124" t="inlineStr">
+        <is>
+          <t>MOB-008</t>
+        </is>
+      </c>
+      <c r="C32" s="125" t="inlineStr">
+        <is>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="D32" s="124" t="inlineStr">
+        <is>
+          <t>El menú administrativo móvil no navega a Remates a 390 px.</t>
+        </is>
+      </c>
+      <c r="E32" s="129" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F32" s="124" t="inlineStr">
+        <is>
+          <t>Corregir la misma transición de navegación móvil de MOB-004 y cubrir los tres destinos y las acciones del menú.</t>
+        </is>
+      </c>
+      <c r="G32" s="124" t="inlineStr">
+        <is>
+          <t>Cada destino, Ver sitio público y Cerrar sesión responden desde el menú móvil.</t>
+        </is>
+      </c>
+      <c r="H32" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I32" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="78" customHeight="1">
+      <c r="A33" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B33" s="124" t="inlineStr">
+        <is>
+          <t>MOB-013</t>
+        </is>
+      </c>
+      <c r="C33" s="125" t="inlineStr">
+        <is>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="D33" s="124" t="inlineStr">
+        <is>
+          <t>Al pasar a escritorio queda visible el control × propio del sidebar móvil.</t>
+        </is>
+      </c>
+      <c r="E33" s="129" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F33" s="124" t="inlineStr">
+        <is>
+          <t>Restablecer explícitamente el estado del sidebar al cruzar el breakpoint y ocultar el control móvil en escritorio.</t>
+        </is>
+      </c>
+      <c r="G33" s="124" t="inlineStr">
+        <is>
+          <t>Tras cambiar de ancho no quedan backdrop, scroll bloqueado ni controles/navegación móviles residuales.</t>
+        </is>
+      </c>
+      <c r="H33" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I33" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="78" customHeight="1">
+      <c r="A34" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B34" s="124" t="inlineStr">
+        <is>
+          <t>MOB-014</t>
+        </is>
+      </c>
+      <c r="C34" s="125" t="inlineStr">
+        <is>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="D34" s="124" t="inlineStr">
+        <is>
+          <t>El editor de remate produce scroll horizontal a 320 y 390 px por el sidebar oculto desplazado.</t>
+        </is>
+      </c>
+      <c r="E34" s="129" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="F34" s="124" t="inlineStr">
+        <is>
+          <t>Sacar el sidebar cerrado del flujo de overflow (por ejemplo, overflow-x:hidden en el contenedor correcto o una estrategia de transform/position que no amplíe el documento) y validar todos los campos.</t>
+        </is>
+      </c>
+      <c r="G34" s="124" t="inlineStr">
+        <is>
+          <t>A 320, 390 y 456 px document.scrollWidth no supera innerWidth y ningún campo, dropzone o botón queda fuera.</t>
+        </is>
+      </c>
+      <c r="H34" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I34" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="78" customHeight="1">
+      <c r="A35" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B35" s="124" t="inlineStr">
+        <is>
+          <t>MOB-015</t>
+        </is>
+      </c>
+      <c r="C35" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D35" s="124" t="inlineStr">
+        <is>
+          <t>No existe fixture con fotografías para validar lightbox móvil.</t>
+        </is>
+      </c>
+      <c r="E35" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F35" s="124" t="inlineStr">
+        <is>
+          <t>Reutilizar o crear el fixture visual propuesto para MOB-003.</t>
+        </is>
+      </c>
+      <c r="G35" s="124" t="inlineStr">
+        <is>
+          <t>La imagen ampliada conserva proporción, aprovecha el teléfono y permite cerrar/navegar.</t>
+        </is>
+      </c>
+      <c r="H35" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I35" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="78" customHeight="1">
+      <c r="A36" s="124" t="inlineStr">
+        <is>
+          <t>Mobile y accesibilidad</t>
+        </is>
+      </c>
+      <c r="B36" s="124" t="inlineStr">
+        <is>
+          <t>ACC-A11Y-006</t>
+        </is>
+      </c>
+      <c r="C36" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D36" s="124" t="inlineStr">
+        <is>
+          <t>La confirmación tiene semántica accesible, pero falta lightbox para completar la cobertura de todos los modales.</t>
+        </is>
+      </c>
+      <c r="E36" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F36" s="124" t="inlineStr">
+        <is>
+          <t>Agregar imágenes al fixture QA y comprobar Escape, foco y restauración de scroll tanto en confirmación como en lightbox.</t>
+        </is>
+      </c>
+      <c r="G36" s="124" t="inlineStr">
+        <is>
+          <t>Cada modal tiene nombre, cierra con Escape y restaura foco y scroll.</t>
+        </is>
+      </c>
+      <c r="H36" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I36" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="78" customHeight="1">
+      <c r="A37" s="124" t="inlineStr">
+        <is>
+          <t>Acceso y sesión</t>
+        </is>
+      </c>
+      <c r="B37" s="124" t="inlineStr">
+        <is>
+          <t>ACC-016</t>
+        </is>
+      </c>
+      <c r="C37" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D37" s="124" t="inlineStr">
+        <is>
+          <t>No hay mecanismo controlado para simular red/API administrativa caída en el Preview.</t>
+        </is>
+      </c>
+      <c r="E37" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F37" s="124" t="inlineStr">
+        <is>
+          <t>Agregar E2E local con route interception/MSW o un flag QA exclusivo de test para responder error y restaurar la API.</t>
+        </is>
+      </c>
+      <c r="G37" s="124" t="inlineStr">
+        <is>
+          <t>El panel ofrece Reintentar y Cerrar sesión y se recupera al restablecer el endpoint.</t>
+        </is>
+      </c>
+      <c r="H37" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I37" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="78" customHeight="1">
+      <c r="A38" s="124" t="inlineStr">
+        <is>
+          <t>Acceso y sesión</t>
+        </is>
+      </c>
+      <c r="B38" s="124" t="inlineStr">
+        <is>
+          <t>ACC-017</t>
+        </is>
+      </c>
+      <c r="C38" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D38" s="124" t="inlineStr">
+        <is>
+          <t>No hay una sesión QA con access token vencido y refresh válido controlable desde el Preview.</t>
+        </is>
+      </c>
+      <c r="E38" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F38" s="124" t="inlineStr">
+        <is>
+          <t>Crear una prueba de integración/E2E que emita o simule tokens con expiración corta y observe una sola repetición de escritura.</t>
+        </is>
+      </c>
+      <c r="G38" s="124" t="inlineStr">
+        <is>
+          <t>Se renueva una vez y la operación genera una única escritura.</t>
+        </is>
+      </c>
+      <c r="H38" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I38" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="78" customHeight="1">
+      <c r="A39" s="124" t="inlineStr">
+        <is>
+          <t>Gestión de remates</t>
+        </is>
+      </c>
+      <c r="B39" s="124" t="inlineStr">
+        <is>
+          <t>REM-026</t>
+        </is>
+      </c>
+      <c r="C39" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D39" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture Finalizado o Cancelado.</t>
+        </is>
+      </c>
+      <c r="E39" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F39" s="124" t="inlineStr">
+        <is>
+          <t>Crear dos remates QA terminales, sin exposición pública, para revisar las acciones disponibles.</t>
+        </is>
+      </c>
+      <c r="G39" s="124" t="inlineStr">
+        <is>
+          <t>Los estados terminales no ofrecen transición a estados activos.</t>
+        </is>
+      </c>
+      <c r="H39" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I39" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="78" customHeight="1">
+      <c r="A40" s="124" t="inlineStr">
+        <is>
+          <t>Gestión de remates</t>
+        </is>
+      </c>
+      <c r="B40" s="124" t="inlineStr">
+        <is>
+          <t>REM-031</t>
+        </is>
+      </c>
+      <c r="C40" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D40" s="124" t="inlineStr">
+        <is>
+          <t>Falta el fixture con fecha Montevideo exacta.</t>
+        </is>
+      </c>
+      <c r="E40" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F40" s="124" t="inlineStr">
+        <is>
+          <t>Crear un fixture QA fechado 30/08/2026 14:30 y comprobarlo antes y después de recargar.</t>
+        </is>
+      </c>
+      <c r="G40" s="124" t="inlineStr">
+        <is>
+          <t>La fecha y hora no sufren corrimiento en panel ni web pública.</t>
+        </is>
+      </c>
+      <c r="H40" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I40" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="78" customHeight="1">
+      <c r="A41" s="124" t="inlineStr">
+        <is>
+          <t>Gestión de remates</t>
+        </is>
+      </c>
+      <c r="B41" s="124" t="inlineStr">
+        <is>
+          <t>REM-040</t>
+        </is>
+      </c>
+      <c r="C41" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D41" s="124" t="inlineStr">
+        <is>
+          <t>No hay remate terminal disponible para editar.</t>
+        </is>
+      </c>
+      <c r="E41" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F41" s="124" t="inlineStr">
+        <is>
+          <t>Reutilizar los fixtures terminales de REM-026 y restaurar cualquier texto modificado.</t>
+        </is>
+      </c>
+      <c r="G41" s="124" t="inlineStr">
+        <is>
+          <t>Editar datos conserva Finalizado o Cancelado y no muestra reactivación.</t>
+        </is>
+      </c>
+      <c r="H41" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I41" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="78" customHeight="1">
+      <c r="A42" s="124" t="inlineStr">
+        <is>
+          <t>Contenido y contacto</t>
+        </is>
+      </c>
+      <c r="B42" s="124" t="inlineStr">
+        <is>
+          <t>CON-006</t>
+        </is>
+      </c>
+      <c r="C42" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D42" s="124" t="inlineStr">
+        <is>
+          <t>No hay simulación de red controlada para el formulario.</t>
+        </is>
+      </c>
+      <c r="E42" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F42" s="124" t="inlineStr">
+        <is>
+          <t>Usar E2E con interceptación de la solicitud de contacto; no enviar correos reales.</t>
+        </is>
+      </c>
+      <c r="G42" s="124" t="inlineStr">
+        <is>
+          <t>El formulario conserva valores y muestra el error al fallar la red.</t>
+        </is>
+      </c>
+      <c r="H42" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I42" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="78" customHeight="1">
+      <c r="A43" s="124" t="inlineStr">
+        <is>
+          <t>Contenido y contacto</t>
+        </is>
+      </c>
+      <c r="B43" s="124" t="inlineStr">
+        <is>
+          <t>CON-016</t>
+        </is>
+      </c>
+      <c r="C43" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D43" s="124" t="inlineStr">
+        <is>
+          <t>No hay simulación controlada del fallo al guardar contenido.</t>
+        </is>
+      </c>
+      <c r="E43" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F43" s="124" t="inlineStr">
+        <is>
+          <t>Interceptar la mutación de contenido en E2E/local y restaurar el estado al finalizar.</t>
+        </is>
+      </c>
+      <c r="G43" s="124" t="inlineStr">
+        <is>
+          <t>Los campos se conservan y la web pública no cambia ante el error.</t>
+        </is>
+      </c>
+      <c r="H43" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I43" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="78" customHeight="1">
+      <c r="A44" s="124" t="inlineStr">
+        <is>
+          <t>Contenido y contacto</t>
+        </is>
+      </c>
+      <c r="B44" s="124" t="inlineStr">
+        <is>
+          <t>CON-018</t>
+        </is>
+      </c>
+      <c r="C44" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D44" s="124" t="inlineStr">
+        <is>
+          <t>El caso requiere persistir cambios públicos de FAQ sin fixture restaurable.</t>
+        </is>
+      </c>
+      <c r="E44" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F44" s="124" t="inlineStr">
+        <is>
+          <t>Crear una configuración de contenido QA aislada o un test E2E transaccional para alta/edición/baja de FAQs.</t>
+        </is>
+      </c>
+      <c r="G44" s="124" t="inlineStr">
+        <is>
+          <t>Las FAQs quedan exactamente guardadas y ordenadas tras recarga.</t>
+        </is>
+      </c>
+      <c r="H44" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I44" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="78" customHeight="1">
+      <c r="A45" s="124" t="inlineStr">
+        <is>
+          <t>API, Supabase y entornos</t>
+        </is>
+      </c>
+      <c r="B45" s="124" t="inlineStr">
+        <is>
+          <t>API-018</t>
+        </is>
+      </c>
+      <c r="C45" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D45" s="124" t="inlineStr">
+        <is>
+          <t>No se puede consultar directamente el contrato público desde este Edge por bloqueo del cliente.</t>
+        </is>
+      </c>
+      <c r="E45" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F45" s="124" t="inlineStr">
+        <is>
+          <t>Ejecutar el contrato en CI o un perfil limpio y validar UTF-8 e instantes ISO contra la zona de Montevideo.</t>
+        </is>
+      </c>
+      <c r="G45" s="124" t="inlineStr">
+        <is>
+          <t>El JSON conserva caracteres y devuelve fechas ISO coherentes.</t>
+        </is>
+      </c>
+      <c r="H45" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I45" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="78" customHeight="1">
+      <c r="A46" s="124" t="inlineStr">
+        <is>
+          <t>API, Supabase y entornos</t>
+        </is>
+      </c>
+      <c r="B46" s="124" t="inlineStr">
+        <is>
+          <t>API-020</t>
+        </is>
+      </c>
+      <c r="C46" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D46" s="124" t="inlineStr">
+        <is>
+          <t>La promoción a main no puede verificarse desde la rama Preview actual.</t>
+        </is>
+      </c>
+      <c r="E46" s="129" t="inlineStr">
+        <is>
+          <t>Proceso de despliegue</t>
+        </is>
+      </c>
+      <c r="F46" s="124" t="inlineStr">
+        <is>
+          <t>Registrar en CI el vínculo entre aprobación de Preview y promoción a main, con historial auditable.</t>
+        </is>
+      </c>
+      <c r="G46" s="124" t="inlineStr">
+        <is>
+          <t>Cada promoción a main referencia un Preview previamente aprobado.</t>
+        </is>
+      </c>
+      <c r="H46" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I46" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="78" customHeight="1">
+      <c r="A47" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B47" s="124" t="inlineStr">
+        <is>
+          <t>CAT-007</t>
+        </is>
+      </c>
+      <c r="C47" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D47" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para persistir una fotografía válida.</t>
+        </is>
+      </c>
+      <c r="E47" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F47" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G47" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H47" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I47" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="78" customHeight="1">
+      <c r="A48" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B48" s="124" t="inlineStr">
+        <is>
+          <t>CAT-008</t>
+        </is>
+      </c>
+      <c r="C48" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D48" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para carrusel con más de tres lotes.</t>
+        </is>
+      </c>
+      <c r="E48" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F48" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G48" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H48" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I48" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="78" customHeight="1">
+      <c r="A49" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B49" s="124" t="inlineStr">
+        <is>
+          <t>CAT-009</t>
+        </is>
+      </c>
+      <c r="C49" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D49" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para bloquear clics repetidos durante transición.</t>
+        </is>
+      </c>
+      <c r="E49" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F49" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G49" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H49" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I49" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="78" customHeight="1">
+      <c r="A50" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B50" s="124" t="inlineStr">
+        <is>
+          <t>CAT-011</t>
+        </is>
+      </c>
+      <c r="C50" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D50" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para rechazar imagen mayor al límite.</t>
+        </is>
+      </c>
+      <c r="E50" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F50" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G50" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H50" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I50" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="78" customHeight="1">
+      <c r="A51" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B51" s="124" t="inlineStr">
+        <is>
+          <t>CAT-012</t>
+        </is>
+      </c>
+      <c r="C51" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D51" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para abrir y cerrar imagen ampliada.</t>
+        </is>
+      </c>
+      <c r="E51" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F51" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G51" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H51" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I51" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="78" customHeight="1">
+      <c r="A52" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B52" s="124" t="inlineStr">
+        <is>
+          <t>CAT-013</t>
+        </is>
+      </c>
+      <c r="C52" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D52" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para arrastrar varias imágenes juntas.</t>
+        </is>
+      </c>
+      <c r="E52" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F52" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G52" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H52" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I52" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="78" customHeight="1">
+      <c r="A53" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B53" s="124" t="inlineStr">
+        <is>
+          <t>CAT-014</t>
+        </is>
+      </c>
+      <c r="C53" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D53" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para exigir nombre por fotografía.</t>
+        </is>
+      </c>
+      <c r="E53" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F53" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G53" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H53" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I53" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="78" customHeight="1">
+      <c r="A54" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B54" s="124" t="inlineStr">
+        <is>
+          <t>CAT-015</t>
+        </is>
+      </c>
+      <c r="C54" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D54" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para impedir lote destacado sin fotografía.</t>
+        </is>
+      </c>
+      <c r="E54" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F54" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G54" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H54" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I54" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="78" customHeight="1">
+      <c r="A55" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B55" s="124" t="inlineStr">
+        <is>
+          <t>CAT-016</t>
+        </is>
+      </c>
+      <c r="C55" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D55" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para rechazar formatos no permitidos o vacíos.</t>
+        </is>
+      </c>
+      <c r="E55" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F55" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G55" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H55" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I55" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="78" customHeight="1">
+      <c r="A56" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B56" s="124" t="inlineStr">
+        <is>
+          <t>CAT-017</t>
+        </is>
+      </c>
+      <c r="C56" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D56" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para rechazar contenido falso o mime incorrecto.</t>
+        </is>
+      </c>
+      <c r="E56" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F56" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G56" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H56" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I56" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="78" customHeight="1">
+      <c r="A57" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B57" s="124" t="inlineStr">
+        <is>
+          <t>CAT-018</t>
+        </is>
+      </c>
+      <c r="C57" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D57" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para máximo de ocho fotografías.</t>
+        </is>
+      </c>
+      <c r="E57" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F57" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G57" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H57" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I57" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="78" customHeight="1">
+      <c r="A58" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B58" s="124" t="inlineStr">
+        <is>
+          <t>CAT-019</t>
+        </is>
+      </c>
+      <c r="C58" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D58" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para selección mixta de archivos.</t>
+        </is>
+      </c>
+      <c r="E58" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F58" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G58" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H58" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I58" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="78" customHeight="1">
+      <c r="A59" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B59" s="124" t="inlineStr">
+        <is>
+          <t>CAT-020</t>
+        </is>
+      </c>
+      <c r="C59" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D59" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para quitar una fotografía existente.</t>
+        </is>
+      </c>
+      <c r="E59" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F59" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G59" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H59" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I59" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="78" customHeight="1">
+      <c r="A60" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B60" s="124" t="inlineStr">
+        <is>
+          <t>CAT-021</t>
+        </is>
+      </c>
+      <c r="C60" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D60" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para eliminar remate con fotografías.</t>
+        </is>
+      </c>
+      <c r="E60" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F60" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G60" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H60" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I60" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="78" customHeight="1">
+      <c r="A61" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B61" s="124" t="inlineStr">
+        <is>
+          <t>CAT-022</t>
+        </is>
+      </c>
+      <c r="C61" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D61" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para renombrar una fotografía.</t>
+        </is>
+      </c>
+      <c r="E61" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F61" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G61" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H61" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I61" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="78" customHeight="1">
+      <c r="A62" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B62" s="124" t="inlineStr">
+        <is>
+          <t>CAT-023</t>
+        </is>
+      </c>
+      <c r="C62" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D62" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para bloquear acceso directo al bucket.</t>
+        </is>
+      </c>
+      <c r="E62" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F62" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G62" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H62" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I62" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="78" customHeight="1">
+      <c r="A63" s="124" t="inlineStr">
+        <is>
+          <t>Catálogo y lotes</t>
+        </is>
+      </c>
+      <c r="B63" s="124" t="inlineStr">
+        <is>
+          <t>CAT-024</t>
+        </is>
+      </c>
+      <c r="C63" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D63" s="124" t="inlineStr">
+        <is>
+          <t>No hay fixture de imagen/lote para renovar url firmada.</t>
+        </is>
+      </c>
+      <c r="E63" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F63" s="124" t="inlineStr">
+        <is>
+          <t>Crear un remate QA aislado con fotografías válidas y una copia local de archivos de borde para toda la suite CAT.</t>
+        </is>
+      </c>
+      <c r="G63" s="124" t="inlineStr">
+        <is>
+          <t>El flujo específico del caso se completa y la limpieza deja Storage sin objetos QA huérfanos.</t>
+        </is>
+      </c>
+      <c r="H63" s="130" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I63" s="128" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="78" customHeight="1">
+      <c r="A64" s="124" t="inlineStr">
+        <is>
+          <t>API, Supabase y entornos</t>
+        </is>
+      </c>
+      <c r="B64" s="124" t="inlineStr">
+        <is>
+          <t>API-019</t>
+        </is>
+      </c>
+      <c r="C64" s="125" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="D64" s="124" t="inlineStr">
+        <is>
+          <t>No se puede comparar Preview y Production dentro del alcance autorizado.</t>
+        </is>
+      </c>
+      <c r="E64" s="129" t="inlineStr">
+        <is>
+          <t>Entorno de prueba</t>
+        </is>
+      </c>
+      <c r="F64" s="124" t="inlineStr">
+        <is>
+          <t>Definir dos entornos QA explícitos o una comprobación CI de configuración que no consulte datos de producción.</t>
+        </is>
+      </c>
+      <c r="G64" s="124" t="inlineStr">
+        <is>
+          <t>La prueba compara identificadores/configuración aprobados y confirma que datos QA no se exponen en producción.</t>
+        </is>
+      </c>
+      <c r="H64" s="130" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I64" s="128" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
@@ -7266,15 +9004,37 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K17" s="44" t="str"/>
-      <c r="L17" s="44" t="str"/>
-      <c r="M17" s="44" t="str"/>
-      <c r="N17" s="44" t="str"/>
-      <c r="O17" s="44" t="str"/>
-      <c r="P17" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>No se dispuso de un modo offline ni de bloqueo controlado del endpoint administrativo en el Preview protegido.</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El control de red no está disponible en esta automatización; no se simuló un fallo real.</t>
+        </is>
+      </c>
+      <c r="M17" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O17" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P17" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="68" customHeight="1">
       <c r="A18" s="51" t="inlineStr">
@@ -7326,15 +9086,37 @@
       </c>
       <c r="J18" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K18" s="50" t="str"/>
-      <c r="L18" s="50" t="str"/>
-      <c r="M18" s="50" t="str"/>
-      <c r="N18" s="50" t="str"/>
-      <c r="O18" s="50" t="str"/>
-      <c r="P18" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K18" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo expirar/controlar el access token conservando un refresh válido en el Preview protegido.</t>
+        </is>
+      </c>
+      <c r="L18" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Requiere fixture de sesión o prueba E2E que controle la expiración sin escribir datos.</t>
+        </is>
+      </c>
+      <c r="M18" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N18" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O18" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P18" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J11">
@@ -8605,19 +10387,38 @@
       </c>
       <c r="J16" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K16" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="inlineStr">
+        <is>
+          <t>Las ayudas contextuales de campos se activan, muestran texto específico y no cubren el input de forma permanente.</t>
+        </is>
+      </c>
       <c r="L16" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Las ayudas de Título, Fecha, Estado del catálogo y Condiciones aparecieron con el mouse y desaparecieron al salir.</t>
-        </is>
-      </c>
-      <c r="M16" s="50" t="str"/>
-      <c r="N16" s="50" t="str"/>
-      <c r="O16" s="50" t="str"/>
-      <c r="P16" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Las ayudas de Título, Fecha, Estado del catálogo y Condiciones aparecieron con el mouse y desaparecieron al salir.
+QA 12/10/2026: Se verificaron 12 ayudas del editor; la del título se mostró con role=tooltip y texto asociado.</t>
+        </is>
+      </c>
+      <c r="M16" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N16" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O16" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P16" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
@@ -8834,19 +10635,37 @@
       </c>
       <c r="J19" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K19" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K19" s="44" t="inlineStr">
+        <is>
+          <t>Se rechazaron texto libre, 31/02/2026 17:00 y 20/06/2026 25:00 con el mensaje de formato requerido; no se publicó remate.</t>
+        </is>
+      </c>
       <c r="L19" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Los tres valores inválidos fueron rechazados con el mensaje de formato dd/mm/yyyy HH:mm. Valores probados: texto libre, 31/02/2026 17:00 y 20/06/2026 25:00.</t>
-        </is>
-      </c>
-      <c r="M19" s="44" t="str"/>
-      <c r="N19" s="44" t="str"/>
-      <c r="O19" s="44" t="str"/>
-      <c r="P19" s="44" t="str"/>
+          <t>QA 12/10/2026: Los tres valores inválidos conservaron el editor y mostraron “Ingresá una fecha válida con el formato dd/mm/yyyy HH:mm”.</t>
+        </is>
+      </c>
+      <c r="M19" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N19" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O19" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P19" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="68" customHeight="1">
       <c r="A20" s="51" t="inlineStr">
@@ -9365,19 +11184,38 @@
       </c>
       <c r="J26" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K26" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K26" s="50" t="inlineStr">
+        <is>
+          <t>No hay remates en estado Finalizado o Cancelado para comprobar que no ofrezcan reactivación.</t>
+        </is>
+      </c>
       <c r="L26" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Finalizado y Cancelado solo ofrecieron Editar y Eliminar; el editor no mostró acciones para reactivarlos.</t>
-        </is>
-      </c>
-      <c r="M26" s="50" t="str"/>
-      <c r="N26" s="50" t="str"/>
-      <c r="O26" s="50" t="str"/>
-      <c r="P26" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Finalizado y Cancelado solo ofrecieron Editar y Eliminar; el editor no mostró acciones para reactivarlos.
+QA 12/10/2026: El listado actual contiene cinco Publicados y cero estados terminales.</t>
+        </is>
+      </c>
+      <c r="M26" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N26" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O26" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P26" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="68" customHeight="1">
       <c r="A27" s="52" t="inlineStr">
@@ -9706,19 +11544,38 @@
       </c>
       <c r="J31" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K31" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K31" s="44" t="inlineStr">
+        <is>
+          <t>No está disponible el fixture con fecha 30/08/2026 14:30 requerido por el caso.</t>
+        </is>
+      </c>
       <c r="L31" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Después de guardar y recargar se mantuvo 30/08/2026 14:30 en editor, listado y detalle.</t>
-        </is>
-      </c>
-      <c r="M31" s="44" t="str"/>
-      <c r="N31" s="44" t="str"/>
-      <c r="O31" s="44" t="str"/>
-      <c r="P31" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Después de guardar y recargar se mantuvo 30/08/2026 14:30 en editor, listado y detalle.
+QA 12/10/2026: El listado actual no incluye ese remate; no se alteraron fechas de datos existentes.</t>
+        </is>
+      </c>
+      <c r="M31" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N31" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O31" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P31" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="68" customHeight="1">
       <c r="A32" s="51" t="inlineStr">
@@ -10379,15 +12236,37 @@
       </c>
       <c r="J40" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K40" s="50" t="str"/>
-      <c r="L40" s="50" t="str"/>
-      <c r="M40" s="50" t="str"/>
-      <c r="N40" s="50" t="str"/>
-      <c r="O40" s="50" t="str"/>
-      <c r="P40" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K40" s="50" t="inlineStr">
+        <is>
+          <t>No hay un remate terminal para editar sin reactivarlo.</t>
+        </is>
+      </c>
+      <c r="L40" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El listado actual tiene cero Finalizados y cero Cancelados.</t>
+        </is>
+      </c>
+      <c r="M40" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N40" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O40" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P40" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="68" customHeight="1">
       <c r="A41" s="52" t="inlineStr">
@@ -10738,19 +12617,38 @@
       </c>
       <c r="J3" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K3" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K3" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar persistir una fotografía válida: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L3" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Se cargaron seis PNG válidos y cada tarjeta mostró su nombre en el detalle público.</t>
-        </is>
-      </c>
-      <c r="M3" s="44" t="str"/>
-      <c r="N3" s="44" t="str"/>
-      <c r="O3" s="44" t="str"/>
-      <c r="P3" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Se cargaron seis PNG válidos y cada tarjeta mostró su nombre en el detalle público.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M3" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N3" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O3" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P3" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="68" customHeight="1">
       <c r="A4" s="51" t="inlineStr">
@@ -10801,19 +12699,38 @@
       </c>
       <c r="J4" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K4" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K4" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar carrusel con más de tres lotes: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L4" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Con seis lotes, ocho avances y ocho retrocesos recorrieron el carrusel circularmente y volvieron al primer lote.</t>
-        </is>
-      </c>
-      <c r="M4" s="50" t="str"/>
-      <c r="N4" s="50" t="str"/>
-      <c r="O4" s="50" t="str"/>
-      <c r="P4" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Con seis lotes, ocho avances y ocho retrocesos recorrieron el carrusel circularmente y volvieron al primer lote.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M4" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N4" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O4" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P4" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="68" customHeight="1">
       <c r="A5" s="52" t="inlineStr">
@@ -10864,19 +12781,38 @@
       </c>
       <c r="J5" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K5" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K5" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar bloquear clics repetidos durante transición: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L5" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Diez clics rápidos dejaron tres tarjetas válidas y el control habilitado luego de estabilizarse.</t>
-        </is>
-      </c>
-      <c r="M5" s="44" t="str"/>
-      <c r="N5" s="44" t="str"/>
-      <c r="O5" s="44" t="str"/>
-      <c r="P5" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. Diez clics rápidos dejaron tres tarjetas válidas y el control habilitado luego de estabilizarse.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M5" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N5" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O5" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P5" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="68" customHeight="1">
       <c r="A6" s="51" t="inlineStr">
@@ -10927,19 +12863,38 @@
       </c>
       <c r="J6" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K6" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar rechazar imagen mayor al límite: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L6" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El PNG de 700.001 bytes mostró el aviso de máximo excedido y no se agregó como lote.</t>
-        </is>
-      </c>
-      <c r="M6" s="50" t="str"/>
-      <c r="N6" s="50" t="str"/>
-      <c r="O6" s="50" t="str"/>
-      <c r="P6" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El PNG de 700.001 bytes mostró el aviso de máximo excedido y no se agregó como lote.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M6" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N6" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O6" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P6" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="68" customHeight="1">
       <c r="A7" s="52" t="inlineStr">
@@ -10991,19 +12946,38 @@
       </c>
       <c r="J7" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K7" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar abrir y cerrar imagen ampliada: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L7" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El lightbox navegó entre lotes y cerró con X, Escape y clic fuera.</t>
-        </is>
-      </c>
-      <c r="M7" s="44" t="str"/>
-      <c r="N7" s="44" t="str"/>
-      <c r="O7" s="44" t="str"/>
-      <c r="P7" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El lightbox navegó entre lotes y cerró con X, Escape y clic fuera.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M7" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N7" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O7" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P7" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="68" customHeight="1">
       <c r="A8" s="51" t="inlineStr">
@@ -11055,19 +13029,38 @@
       </c>
       <c r="J8" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K8" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K8" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar arrastrar varias imágenes juntas: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L8" s="50" t="inlineStr">
         <is>
-          <t>La automatización no puede arrastrar archivos desde el sistema operativo. La carga múltiple por selector se verificó en CAT-007.</t>
-        </is>
-      </c>
-      <c r="M8" s="50" t="str"/>
-      <c r="N8" s="50" t="str"/>
-      <c r="O8" s="50" t="str"/>
-      <c r="P8" s="50" t="str"/>
+          <t>La automatización no puede arrastrar archivos desde el sistema operativo. La carga múltiple por selector se verificó en CAT-007.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M8" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N8" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O8" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P8" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="68" customHeight="1">
       <c r="A9" s="52" t="inlineStr">
@@ -11119,19 +13112,38 @@
       </c>
       <c r="J9" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K9" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K9" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar exigir nombre por fotografía: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L9" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El guardado se bloqueó hasta completar el nombre de cada una de las seis imágenes.</t>
-        </is>
-      </c>
-      <c r="M9" s="44" t="str"/>
-      <c r="N9" s="44" t="str"/>
-      <c r="O9" s="44" t="str"/>
-      <c r="P9" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Coincide con el resultado esperado. El guardado se bloqueó hasta completar el nombre de cada una de las seis imágenes.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M9" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N9" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O9" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P9" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="68" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
@@ -11183,19 +13195,38 @@
       </c>
       <c r="J10" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar impedir lote destacado sin fotografía: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
       <c r="L10" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Fallido): No coincide con el resultado esperado. No existe una acción para crear un lote sin fotografía: cada lote se genera únicamente al cargar una imagen.</t>
-        </is>
-      </c>
-      <c r="M10" s="50" t="str"/>
-      <c r="N10" s="50" t="str"/>
-      <c r="O10" s="50" t="str"/>
-      <c r="P10" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Fallido): No coincide con el resultado esperado. No existe una acción para crear un lote sin fotografía: cada lote se genera únicamente al cargar una imagen.
+QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M10" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N10" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="68" customHeight="1">
       <c r="A11" s="52" t="inlineStr">
@@ -11246,15 +13277,37 @@
       </c>
       <c r="J11" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K11" s="44" t="str"/>
-      <c r="L11" s="44" t="str"/>
-      <c r="M11" s="44" t="str"/>
-      <c r="N11" s="44" t="str"/>
-      <c r="O11" s="44" t="str"/>
-      <c r="P11" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K11" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar rechazar formatos no permitidos o vacíos: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L11" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M11" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O11" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P11" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="68" customHeight="1">
       <c r="A12" s="51" t="inlineStr">
@@ -11306,15 +13359,37 @@
       </c>
       <c r="J12" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K12" s="50" t="str"/>
-      <c r="L12" s="50" t="str"/>
-      <c r="M12" s="50" t="str"/>
-      <c r="N12" s="50" t="str"/>
-      <c r="O12" s="50" t="str"/>
-      <c r="P12" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K12" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar rechazar contenido falso o mime incorrecto: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L12" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M12" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N12" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O12" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P12" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="68" customHeight="1">
       <c r="A13" s="52" t="inlineStr">
@@ -11366,15 +13441,37 @@
       </c>
       <c r="J13" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K13" s="44" t="str"/>
-      <c r="L13" s="44" t="str"/>
-      <c r="M13" s="44" t="str"/>
-      <c r="N13" s="44" t="str"/>
-      <c r="O13" s="44" t="str"/>
-      <c r="P13" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K13" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar máximo de ocho fotografías: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L13" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M13" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N13" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O13" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P13" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="68" customHeight="1">
       <c r="A14" s="51" t="inlineStr">
@@ -11425,15 +13522,37 @@
       </c>
       <c r="J14" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K14" s="50" t="str"/>
-      <c r="L14" s="50" t="str"/>
-      <c r="M14" s="50" t="str"/>
-      <c r="N14" s="50" t="str"/>
-      <c r="O14" s="50" t="str"/>
-      <c r="P14" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K14" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar selección mixta de archivos: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L14" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M14" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N14" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O14" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P14" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="68" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
@@ -11485,15 +13604,37 @@
       </c>
       <c r="J15" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K15" s="44" t="str"/>
-      <c r="L15" s="44" t="str"/>
-      <c r="M15" s="44" t="str"/>
-      <c r="N15" s="44" t="str"/>
-      <c r="O15" s="44" t="str"/>
-      <c r="P15" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K15" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar quitar una fotografía existente: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L15" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M15" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N15" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O15" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P15" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="68" customHeight="1">
       <c r="A16" s="51" t="inlineStr">
@@ -11544,15 +13685,37 @@
       </c>
       <c r="J16" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K16" s="50" t="str"/>
-      <c r="L16" s="50" t="str"/>
-      <c r="M16" s="50" t="str"/>
-      <c r="N16" s="50" t="str"/>
-      <c r="O16" s="50" t="str"/>
-      <c r="P16" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar eliminar remate con fotografías: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L16" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M16" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N16" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O16" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P16" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
@@ -11604,15 +13767,37 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K17" s="44" t="str"/>
-      <c r="L17" s="44" t="str"/>
-      <c r="M17" s="44" t="str"/>
-      <c r="N17" s="44" t="str"/>
-      <c r="O17" s="44" t="str"/>
-      <c r="P17" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar renombrar una fotografía: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M17" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O17" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P17" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="68" customHeight="1">
       <c r="A18" s="51" t="inlineStr">
@@ -11663,15 +13848,37 @@
       </c>
       <c r="J18" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K18" s="50" t="str"/>
-      <c r="L18" s="50" t="str"/>
-      <c r="M18" s="50" t="str"/>
-      <c r="N18" s="50" t="str"/>
-      <c r="O18" s="50" t="str"/>
-      <c r="P18" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K18" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar bloquear acceso directo al bucket: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L18" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M18" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N18" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O18" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P18" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="68" customHeight="1">
       <c r="A19" s="52" t="inlineStr">
@@ -11723,15 +13930,37 @@
       </c>
       <c r="J19" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K19" s="44" t="str"/>
-      <c r="L19" s="44" t="str"/>
-      <c r="M19" s="44" t="str"/>
-      <c r="N19" s="44" t="str"/>
-      <c r="O19" s="44" t="str"/>
-      <c r="P19" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K19" s="44" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar renovar url firmada: no hay lote/fotografía QA disponible.</t>
+        </is>
+      </c>
+      <c r="L19" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El remate QA abierto no tiene imágenes, lotes destacados ni URL firmada para ejercer el flujo.</t>
+        </is>
+      </c>
+      <c r="M19" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N19" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O19" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P19" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J11">
@@ -14076,15 +16305,37 @@
       </c>
       <c r="J6" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K6" s="50" t="str"/>
-      <c r="L6" s="50" t="str"/>
-      <c r="M6" s="50" t="str"/>
-      <c r="N6" s="50" t="str"/>
-      <c r="O6" s="50" t="str"/>
-      <c r="P6" s="50" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="inlineStr">
+        <is>
+          <t>El envío no mostró confirmación ni limpió los campos; nombre, email y mensaje permanecieron cargados.</t>
+        </is>
+      </c>
+      <c r="L6" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se intentó enviar una consulta QA autorizada. No hubo role=alert/status ni evidencia de entrega.</t>
+        </is>
+      </c>
+      <c r="M6" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N6" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O6" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P6" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="68" customHeight="1">
       <c r="A7" s="52" t="inlineStr">
@@ -14139,15 +16390,37 @@
       </c>
       <c r="J7" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K7" s="44" t="str"/>
-      <c r="L7" s="44" t="str"/>
-      <c r="M7" s="44" t="str"/>
-      <c r="N7" s="44" t="str"/>
-      <c r="O7" s="44" t="str"/>
-      <c r="P7" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>El Preview no permite simular una caída de red del envío sin emitir una consulta real.</t>
+        </is>
+      </c>
+      <c r="L7" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: No se envió correo ni se alteraron datos del formulario.</t>
+        </is>
+      </c>
+      <c r="M7" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N7" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O7" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P7" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="68" customHeight="1">
       <c r="A8" s="51" t="inlineStr">
@@ -14281,15 +16554,37 @@
       </c>
       <c r="J9" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K9" s="44" t="str"/>
-      <c r="L9" s="44" t="str"/>
-      <c r="M9" s="44" t="str"/>
-      <c r="N9" s="44" t="str"/>
-      <c r="O9" s="44" t="str"/>
-      <c r="P9" s="44" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K9" s="44" t="inlineStr">
+        <is>
+          <t>Las FAQs se guardaron, pero los cambios válidos de contacto y ubicación no se reflejaron tras recargar la web pública.</t>
+        </is>
+      </c>
+      <c r="L9" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Reprueba posterior a la corrección de guardado de FAQ. Persistieron las FAQs, pero email, teléfono, dirección, horario y descripción de ubicación volvieron a sus valores anteriores.</t>
+        </is>
+      </c>
+      <c r="M9" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N9" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O9" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P9" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="68" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
@@ -14344,15 +16639,37 @@
       </c>
       <c r="J10" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="str"/>
-      <c r="L10" s="50" t="str"/>
-      <c r="M10" s="50" t="str"/>
-      <c r="N10" s="50" t="str"/>
-      <c r="O10" s="50" t="str"/>
-      <c r="P10" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>La FAQ temporal se agregó, editó y apareció en la web pública; luego se eliminó como limpieza.</t>
+        </is>
+      </c>
+      <c r="L10" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se verificó publicación y edición desde el panel, seguida de eliminación del fixture.</t>
+        </is>
+      </c>
+      <c r="M10" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N10" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="68" customHeight="1">
       <c r="A11" s="52" t="inlineStr">
@@ -14404,15 +16721,37 @@
       </c>
       <c r="J11" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K11" s="44" t="str"/>
-      <c r="L11" s="44" t="str"/>
-      <c r="M11" s="44" t="str"/>
-      <c r="N11" s="44" t="str"/>
-      <c r="O11" s="44" t="str"/>
-      <c r="P11" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K11" s="44" t="inlineStr">
+        <is>
+          <t>Las FAQs QA temporales se eliminaron, se guardó el cambio y no reaparecieron tras recargar.</t>
+        </is>
+      </c>
+      <c r="L11" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Limpieza confirmada tanto en administrador como en web pública.</t>
+        </is>
+      </c>
+      <c r="M11" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O11" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P11" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="68" customHeight="1">
       <c r="A12" s="51" t="inlineStr">
@@ -14551,12 +16890,12 @@
       </c>
       <c r="K13" s="44" t="inlineStr">
         <is>
-          <t>El guardado de email, teléfono, dirección y horario QA no persistió; la configuración pública mantuvo todos sus valores anteriores.</t>
+          <t>Los cuatro datos temporales de contacto no persistieron: la web conservó los valores previos.</t>
         </is>
       </c>
       <c r="L13" s="44" t="inlineStr">
         <is>
-          <t>QA 12/10/2026: Incidencia: Guardar cambios no aplicó modificaciones válidas en datos públicos de contacto.</t>
+          <t>QA 12/10/2026: Tras guardar y recargar, email, teléfono, dirección y horario públicos continuaron sin cambios.</t>
         </is>
       </c>
       <c r="M13" s="132" t="n">
@@ -14574,7 +16913,7 @@
       </c>
       <c r="P13" s="44" t="inlineStr">
         <is>
-          <t>42f44e1</t>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
         </is>
       </c>
     </row>
@@ -14791,15 +17130,37 @@
       </c>
       <c r="J16" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K16" s="50" t="str"/>
-      <c r="L16" s="50" t="str"/>
-      <c r="M16" s="50" t="str"/>
-      <c r="N16" s="50" t="str"/>
-      <c r="O16" s="50" t="str"/>
-      <c r="P16" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="inlineStr">
+        <is>
+          <t>Un título temporal junto a email inválido no produjo cambios parciales; tras recargar se recuperó el contenido persistido.</t>
+        </is>
+      </c>
+      <c r="L16" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se verificó la atomicidad mediante recarga del panel.</t>
+        </is>
+      </c>
+      <c r="M16" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N16" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O16" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P16" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
@@ -14851,15 +17212,37 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K17" s="44" t="str"/>
-      <c r="L17" s="44" t="str"/>
-      <c r="M17" s="44" t="str"/>
-      <c r="N17" s="44" t="str"/>
-      <c r="O17" s="44" t="str"/>
-      <c r="P17" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>No hay mecanismo de fallo controlado para el guardado de contenido en el Preview.</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se evitó guardar cambios públicos sin una simulación aislada.</t>
+        </is>
+      </c>
+      <c r="M17" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O17" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P17" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="68" customHeight="1">
       <c r="A18" s="51" t="inlineStr">
@@ -14910,15 +17293,37 @@
       </c>
       <c r="J18" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K18" s="50" t="str"/>
-      <c r="L18" s="50" t="str"/>
-      <c r="M18" s="50" t="str"/>
-      <c r="N18" s="50" t="str"/>
-      <c r="O18" s="50" t="str"/>
-      <c r="P18" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K18" s="50" t="inlineStr">
+        <is>
+          <t>Los cuatro pasos públicos se mantienen en su orden: Revisá, Registrate, Participá y Pagos y retiro.</t>
+        </is>
+      </c>
+      <c r="L18" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Comprobado en la home sin editar contenido.</t>
+        </is>
+      </c>
+      <c r="M18" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N18" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O18" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P18" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="68" customHeight="1">
       <c r="A19" s="52" t="inlineStr">
@@ -14970,15 +17375,37 @@
       </c>
       <c r="J19" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K19" s="44" t="str"/>
-      <c r="L19" s="44" t="str"/>
-      <c r="M19" s="44" t="str"/>
-      <c r="N19" s="44" t="str"/>
-      <c r="O19" s="44" t="str"/>
-      <c r="P19" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K19" s="44" t="inlineStr">
+        <is>
+          <t>En un único guardado se agregó, editó y eliminó FAQ; el orden final fue correcto y los fixtures quedaron eliminados.</t>
+        </is>
+      </c>
+      <c r="L19" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Publicación y limpieza verificadas con recarga.</t>
+        </is>
+      </c>
+      <c r="M19" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N19" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O19" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P19" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="68" customHeight="1">
       <c r="A20" s="51" t="inlineStr">
@@ -15034,12 +17461,12 @@
       </c>
       <c r="K20" s="50" t="inlineStr">
         <is>
-          <t>El texto con Ñ, &amp;, comillas y salto de línea no se persistió en la descripción de ubicación.</t>
+          <t>El texto temporal con ñ, &amp;, comillas y salto de línea no se reflejó en la web pública.</t>
         </is>
       </c>
       <c r="L20" s="50" t="inlineStr">
         <is>
-          <t>QA 12/10/2026: Incidencia: el mismo guardado de contenido no confirmó ni aplicó cambios válidos.</t>
+          <t>QA 12/10/2026: El panel mostró los valores locales, pero tras recargar volvieron los persistidos y la web mantuvo el texto anterior.</t>
         </is>
       </c>
       <c r="M20" s="131" t="n">
@@ -15057,7 +17484,7 @@
       </c>
       <c r="P20" s="50" t="inlineStr">
         <is>
-          <t>42f44e1</t>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
         </is>
       </c>
     </row>
@@ -15115,12 +17542,12 @@
       </c>
       <c r="K21" s="44" t="inlineStr">
         <is>
-          <t>La dirección temporal no se persistió, por lo que el enlace externo de Google Maps no pudo reflejarla.</t>
+          <t>La dirección temporal no persistió, por lo que el enlace externo mantuvo la dirección anterior.</t>
         </is>
       </c>
       <c r="L21" s="44" t="inlineStr">
         <is>
-          <t>QA 12/10/2026: Incidencia: el guardado de contenido no actualiza la dirección pública.</t>
+          <t>QA 12/10/2026: La web y el enlace de Google Maps conservaron Av. 18 de Julio 1234, Centro, Montevideo.</t>
         </is>
       </c>
       <c r="M21" s="132" t="n">
@@ -15138,7 +17565,7 @@
       </c>
       <c r="P21" s="44" t="inlineStr">
         <is>
-          <t>42f44e1</t>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
         </is>
       </c>
     </row>
@@ -15325,15 +17752,37 @@
       </c>
       <c r="J2" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K2" s="50" t="str"/>
-      <c r="L2" s="50" t="str"/>
-      <c r="M2" s="50" t="str"/>
-      <c r="N2" s="50" t="str"/>
-      <c r="O2" s="50" t="str"/>
-      <c r="P2" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K2" s="50" t="inlineStr">
+        <is>
+          <t>Home a 320×568 sin scroll horizontal global ni controles fuera de pantalla.</t>
+        </is>
+      </c>
+      <c r="L2" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Recorrido responsive de home; ancho de documento 305 px para viewport de 320 px.</t>
+        </is>
+      </c>
+      <c r="M2" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N2" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O2" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P2" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="68" customHeight="1">
       <c r="A3" s="52" t="inlineStr">
@@ -15385,15 +17834,37 @@
       </c>
       <c r="J3" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K3" s="44" t="str"/>
-      <c r="L3" s="44" t="str"/>
-      <c r="M3" s="44" t="str"/>
-      <c r="N3" s="44" t="str"/>
-      <c r="O3" s="44" t="str"/>
-      <c r="P3" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K3" s="44" t="inlineStr">
+        <is>
+          <t>Home a 390×844: el menú se abrió y la navegación llevó a #contacto sin desborde global.</t>
+        </is>
+      </c>
+      <c r="L3" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Verificado viewport 390 px; document.scrollWidth=375 px y URL final #contacto.</t>
+        </is>
+      </c>
+      <c r="M3" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N3" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O3" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P3" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="68" customHeight="1">
       <c r="A4" s="51" t="inlineStr">
@@ -15445,15 +17916,37 @@
       </c>
       <c r="J4" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K4" s="50" t="str"/>
-      <c r="L4" s="50" t="str"/>
-      <c r="M4" s="50" t="str"/>
-      <c r="N4" s="50" t="str"/>
-      <c r="O4" s="50" t="str"/>
-      <c r="P4" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K4" s="50" t="inlineStr">
+        <is>
+          <t>No se pudo ejecutar el carrusel ni lightbox: el remate QA disponible no tiene lotes ni imágenes.</t>
+        </is>
+      </c>
+      <c r="L4" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Fixture actual: QA paquete actualizado 2026, catálogo sin lotes destacados.</t>
+        </is>
+      </c>
+      <c r="M4" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N4" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O4" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P4" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="68" customHeight="1">
       <c r="A5" s="52" t="inlineStr">
@@ -15505,15 +17998,37 @@
       </c>
       <c r="J5" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K5" s="44" t="str"/>
-      <c r="L5" s="44" t="str"/>
-      <c r="M5" s="44" t="str"/>
-      <c r="N5" s="44" t="str"/>
-      <c r="O5" s="44" t="str"/>
-      <c r="P5" s="44" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K5" s="44" t="inlineStr">
+        <is>
+          <t>A 390×844, al seleccionar Remates desde el menú móvil el panel permaneció en Resumen.</t>
+        </is>
+      </c>
+      <c r="L5" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: La navegación móvil no cambia de sección; impide completar el recorrido Resumen/Remates/editor.</t>
+        </is>
+      </c>
+      <c r="M5" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N5" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O5" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P5" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="68" customHeight="1">
       <c r="A6" s="51" t="inlineStr">
@@ -15564,15 +18079,37 @@
       </c>
       <c r="J6" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K6" s="50" t="str"/>
-      <c r="L6" s="50" t="str"/>
-      <c r="M6" s="50" t="str"/>
-      <c r="N6" s="50" t="str"/>
-      <c r="O6" s="50" t="str"/>
-      <c r="P6" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="inlineStr">
+        <is>
+          <t>Escape cerró el menú móvil y el control volvió a anunciar Abrir menú.</t>
+        </is>
+      </c>
+      <c r="L6" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Comprobado con menú público abierto a menos de 900 px.</t>
+        </is>
+      </c>
+      <c r="M6" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N6" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O6" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P6" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="68" customHeight="1">
       <c r="A7" s="52" t="inlineStr">
@@ -15623,15 +18160,37 @@
       </c>
       <c r="J7" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K7" s="44" t="str"/>
-      <c r="L7" s="44" t="str"/>
-      <c r="M7" s="44" t="str"/>
-      <c r="N7" s="44" t="str"/>
-      <c r="O7" s="44" t="str"/>
-      <c r="P7" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>Al pasar de 800 a 1024 px se cerró el estado móvil y apareció la navegación de escritorio.</t>
+        </is>
+      </c>
+      <c r="L7" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: aria-expanded volvió a false y quedaron visibles los enlaces de escritorio.</t>
+        </is>
+      </c>
+      <c r="M7" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N7" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O7" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P7" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="68" customHeight="1">
       <c r="A8" s="51" t="inlineStr">
@@ -15682,15 +18241,37 @@
       </c>
       <c r="J8" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K8" s="50" t="str"/>
-      <c r="L8" s="50" t="str"/>
-      <c r="M8" s="50" t="str"/>
-      <c r="N8" s="50" t="str"/>
-      <c r="O8" s="50" t="str"/>
-      <c r="P8" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K8" s="50" t="inlineStr">
+        <is>
+          <t>La automatización disponible no permite cambiar el zoom real del navegador al 200%.</t>
+        </is>
+      </c>
+      <c r="L8" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El control de viewport no emula zoom de navegador; requiere verificación manual o E2E/CDP.</t>
+        </is>
+      </c>
+      <c r="M8" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N8" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O8" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P8" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="68" customHeight="1">
       <c r="A9" s="52" t="inlineStr">
@@ -15741,15 +18322,37 @@
       </c>
       <c r="J9" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K9" s="44" t="str"/>
-      <c r="L9" s="44" t="str"/>
-      <c r="M9" s="44" t="str"/>
-      <c r="N9" s="44" t="str"/>
-      <c r="O9" s="44" t="str"/>
-      <c r="P9" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K9" s="44" t="inlineStr">
+        <is>
+          <t>La automatización disponible no permite aplicar prefers-reduced-motion: reduce.</t>
+        </is>
+      </c>
+      <c r="L9" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Requiere DevTools/emulación de media feature o una prueba E2E con esa preferencia.</t>
+        </is>
+      </c>
+      <c r="M9" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N9" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O9" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P9" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="68" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
@@ -15801,15 +18404,37 @@
       </c>
       <c r="J10" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="str"/>
-      <c r="L10" s="50" t="str"/>
-      <c r="M10" s="50" t="str"/>
-      <c r="N10" s="50" t="str"/>
-      <c r="O10" s="50" t="str"/>
-      <c r="P10" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>Home y panel a 2560×1440 no presentaron scroll horizontal ni zonas fuera del viewport.</t>
+        </is>
+      </c>
+      <c r="L10" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Home: ancho útil 2545 px; panel: main 2560 px y sin desborde horizontal.</t>
+        </is>
+      </c>
+      <c r="M10" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N10" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="68" customHeight="1">
       <c r="A11" s="52" t="inlineStr">
@@ -15860,15 +18485,37 @@
       </c>
       <c r="J11" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K11" s="44" t="str"/>
-      <c r="L11" s="44" t="str"/>
-      <c r="M11" s="44" t="str"/>
-      <c r="N11" s="44" t="str"/>
-      <c r="O11" s="44" t="str"/>
-      <c r="P11" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K11" s="44" t="inlineStr">
+        <is>
+          <t>Home a 456×918 sin scroll horizontal global ni contenido mayor que el viewport.</t>
+        </is>
+      </c>
+      <c r="L11" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: document.scrollWidth=441 px para viewport 456 px.</t>
+        </is>
+      </c>
+      <c r="M11" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O11" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P11" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="68" customHeight="1">
       <c r="A12" s="51" t="inlineStr">
@@ -15921,15 +18568,37 @@
       </c>
       <c r="J12" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K12" s="50" t="str"/>
-      <c r="L12" s="50" t="str"/>
-      <c r="M12" s="50" t="str"/>
-      <c r="N12" s="50" t="str"/>
-      <c r="O12" s="50" t="str"/>
-      <c r="P12" s="50" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K12" s="50" t="inlineStr">
+        <is>
+          <t>El menú administrativo móvil se muestra, pero al elegir Remates no cambia desde Resumen a 390×844.</t>
+        </is>
+      </c>
+      <c r="L12" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: La acción de navegación queda sin efecto; no se validaron las demás acciones desde el flujo móvil.</t>
+        </is>
+      </c>
+      <c r="M12" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N12" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O12" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P12" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="68" customHeight="1">
       <c r="A13" s="52" t="inlineStr">
@@ -15980,15 +18649,37 @@
       </c>
       <c r="J13" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K13" s="44" t="str"/>
-      <c r="L13" s="44" t="str"/>
-      <c r="M13" s="44" t="str"/>
-      <c r="N13" s="44" t="str"/>
-      <c r="O13" s="44" t="str"/>
-      <c r="P13" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K13" s="44" t="inlineStr">
+        <is>
+          <t>A 320, 390 y 456 px las tarjetas/listado mostraron completas y pulsables las acciones Editar, Ocultar, Finalizar, Cancelar y Eliminar.</t>
+        </is>
+      </c>
+      <c r="L13" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Sin controles con borde fuera del ancho de cada viewport.</t>
+        </is>
+      </c>
+      <c r="M13" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N13" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O13" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P13" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="68" customHeight="1">
       <c r="A14" s="51" t="inlineStr">
@@ -16039,15 +18730,37 @@
       </c>
       <c r="J14" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K14" s="50" t="str"/>
-      <c r="L14" s="50" t="str"/>
-      <c r="M14" s="50" t="str"/>
-      <c r="N14" s="50" t="str"/>
-      <c r="O14" s="50" t="str"/>
-      <c r="P14" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K14" s="50" t="inlineStr">
+        <is>
+          <t>El editor de FAQ mantuvo inputs y textareas dentro del ancho a 320 y 456 px.</t>
+        </is>
+      </c>
+      <c r="L14" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Sin recortes ni scroll horizontal global; 11 inputs y 9 áreas de texto revisados.</t>
+        </is>
+      </c>
+      <c r="M14" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N14" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O14" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P14" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="68" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
@@ -16098,15 +18811,37 @@
       </c>
       <c r="J15" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K15" s="44" t="str"/>
-      <c r="L15" s="44" t="str"/>
-      <c r="M15" s="44" t="str"/>
-      <c r="N15" s="44" t="str"/>
-      <c r="O15" s="44" t="str"/>
-      <c r="P15" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K15" s="44" t="inlineStr">
+        <is>
+          <t>Los modales de Eliminar, Finalizar y Cancelar a 320 px caben en pantalla, bloquean el scroll de fondo y se cierran con Volver.</t>
+        </is>
+      </c>
+      <c r="L15" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Diálogos con aria-labelledby/aria-describedby, ancho máximo 296 px; no se confirmó ninguna acción.</t>
+        </is>
+      </c>
+      <c r="M15" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N15" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O15" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P15" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="68" customHeight="1">
       <c r="A16" s="51" t="inlineStr">
@@ -16157,15 +18892,37 @@
       </c>
       <c r="J16" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K16" s="50" t="str"/>
-      <c r="L16" s="50" t="str"/>
-      <c r="M16" s="50" t="str"/>
-      <c r="N16" s="50" t="str"/>
-      <c r="O16" s="50" t="str"/>
-      <c r="P16" s="50" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="inlineStr">
+        <is>
+          <t>Tras ampliar a 1024 px quedó visible el botón × del sidebar móvil, aunque no había backdrop.</t>
+        </is>
+      </c>
+      <c r="L16" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Persistió estado residual de navegación móvil al cambiar de ancho.</t>
+        </is>
+      </c>
+      <c r="M16" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N16" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O16" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P16" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
@@ -16216,15 +18973,37 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K17" s="44" t="str"/>
-      <c r="L17" s="44" t="str"/>
-      <c r="M17" s="44" t="str"/>
-      <c r="N17" s="44" t="str"/>
-      <c r="O17" s="44" t="str"/>
-      <c r="P17" s="44" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>El editor de remate desborda horizontalmente a 320 y 390 px.</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: document.scrollWidth=377 px a 320 y 409 px a 390; el sidebar oculto desplazado contribuye al desborde.</t>
+        </is>
+      </c>
+      <c r="M17" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O17" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P17" s="44" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="68" customHeight="1">
       <c r="A18" s="51" t="inlineStr">
@@ -16276,15 +19055,37 @@
       </c>
       <c r="J18" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K18" s="50" t="str"/>
-      <c r="L18" s="50" t="str"/>
-      <c r="M18" s="50" t="str"/>
-      <c r="N18" s="50" t="str"/>
-      <c r="O18" s="50" t="str"/>
-      <c r="P18" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K18" s="50" t="inlineStr">
+        <is>
+          <t>No hay fotografías/lotes en el fixture QA para abrir la imagen a pantalla completa.</t>
+        </is>
+      </c>
+      <c r="L18" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El detalle QA disponible no expone imágenes ni controles de lightbox.</t>
+        </is>
+      </c>
+      <c r="M18" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N18" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O18" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P18" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="68" customHeight="1">
       <c r="A19" s="52" t="inlineStr">
@@ -16418,15 +19219,37 @@
       </c>
       <c r="J20" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K20" s="50" t="str"/>
-      <c r="L20" s="50" t="str"/>
-      <c r="M20" s="50" t="str"/>
-      <c r="N20" s="50" t="str"/>
-      <c r="O20" s="50" t="str"/>
-      <c r="P20" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K20" s="50" t="inlineStr">
+        <is>
+          <t>El modal de confirmación sí tiene nombre y descripción accesibles, pero no hay lightbox para completar el caso sobre todos los modales.</t>
+        </is>
+      </c>
+      <c r="L20" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Confirmación: aria-labelledby=admin-confirm-title y aria-describedby=admin-confirm-description; falta fixture con imagen.</t>
+        </is>
+      </c>
+      <c r="M20" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N20" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O20" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P20" s="50" t="inlineStr">
+        <is>
+          <t>42f44e1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="J2:J12">
@@ -17010,7 +19833,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="66" t="inlineStr">
         <is>
@@ -17834,15 +20656,37 @@
       </c>
       <c r="J10" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="str"/>
-      <c r="L10" s="50" t="str"/>
-      <c r="M10" s="50" t="str"/>
-      <c r="N10" s="50" t="str"/>
-      <c r="O10" s="50" t="str"/>
-      <c r="P10" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>La sesión pública no expone claves en localStorage ni sessionStorage.</t>
+        </is>
+      </c>
+      <c r="L10" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Dos sesiones públicas mostraron ambos almacenamientos vacíos.</t>
+        </is>
+      </c>
+      <c r="M10" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N10" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="68" customHeight="1">
       <c r="A11" s="52" t="inlineStr">
@@ -17894,15 +20738,37 @@
       </c>
       <c r="J11" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K11" s="44" t="str"/>
-      <c r="L11" s="44" t="str"/>
-      <c r="M11" s="44" t="str"/>
-      <c r="N11" s="44" t="str"/>
-      <c r="O11" s="44" t="str"/>
-      <c r="P11" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K11" s="44" t="inlineStr">
+        <is>
+          <t>Dos sesiones independientes mostraron exactamente la misma lista pública, incluido el remate QA.</t>
+        </is>
+      </c>
+      <c r="L11" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Comparación de contenido tras cargar ambas sesiones.</t>
+        </is>
+      </c>
+      <c r="M11" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O11" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P11" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="68" customHeight="1">
       <c r="A12" s="51" t="inlineStr">
@@ -18307,15 +21173,37 @@
       </c>
       <c r="J18" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K18" s="50" t="str"/>
-      <c r="L18" s="50" t="str"/>
-      <c r="M18" s="50" t="str"/>
-      <c r="N18" s="50" t="str"/>
-      <c r="O18" s="50" t="str"/>
-      <c r="P18" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K18" s="50" t="inlineStr">
+        <is>
+          <t>Un cambio válido acompañado de una FAQ sin respuesta no dejó actualización parcial tras recargar.</t>
+        </is>
+      </c>
+      <c r="L18" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se cargó título temporal y FAQ incompleta. No hubo confirmación de éxito y, tras recargar, no persistieron ni el título ni la FAQ.</t>
+        </is>
+      </c>
+      <c r="M18" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N18" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O18" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P18" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a (Preview; migración DB QA sin commit)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="68" customHeight="1">
       <c r="A19" s="52" t="inlineStr">
@@ -18366,15 +21254,37 @@
       </c>
       <c r="J19" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K19" s="44" t="str"/>
-      <c r="L19" s="44" t="str"/>
-      <c r="M19" s="44" t="str"/>
-      <c r="N19" s="44" t="str"/>
-      <c r="O19" s="44" t="str"/>
-      <c r="P19" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K19" s="44" t="inlineStr">
+        <is>
+          <t>La interfaz conserva UTF-8, pero no se pudo comprobar el contrato API de fechas ISO porque el navegador bloquea la consulta directa.</t>
+        </is>
+      </c>
+      <c r="L19" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: Se visualizó correctamente Ñ, &amp;, 12,5% y comillas en el remate QA.</t>
+        </is>
+      </c>
+      <c r="M19" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N19" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O19" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P19" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="68" customHeight="1">
       <c r="A20" s="51" t="inlineStr">
@@ -18425,15 +21335,37 @@
       </c>
       <c r="J20" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K20" s="50" t="str"/>
-      <c r="L20" s="50" t="str"/>
-      <c r="M20" s="50" t="str"/>
-      <c r="N20" s="50" t="str"/>
-      <c r="O20" s="50" t="str"/>
-      <c r="P20" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K20" s="50" t="inlineStr">
+        <is>
+          <t>No se comparó contra Production: esta ejecución está acotada al Preview protegido.</t>
+        </is>
+      </c>
+      <c r="L20" s="50" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: El alcance prohíbe probar silenciosamente contra producción; no hay evidencia de configuración cruzada.</t>
+        </is>
+      </c>
+      <c r="M20" s="131" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N20" s="50" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O20" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P20" s="50" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="68" customHeight="1">
       <c r="A21" s="52" t="inlineStr">
@@ -18485,15 +21417,37 @@
       </c>
       <c r="J21" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K21" s="44" t="str"/>
-      <c r="L21" s="44" t="str"/>
-      <c r="M21" s="44" t="str"/>
-      <c r="N21" s="44" t="str"/>
-      <c r="O21" s="44" t="str"/>
-      <c r="P21" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K21" s="44" t="inlineStr">
+        <is>
+          <t>La rama actual es codex/nuevo-diseno-home y no hay evidencia de una promoción controlada a main en esta ejecución.</t>
+        </is>
+      </c>
+      <c r="L21" s="44" t="inlineStr">
+        <is>
+          <t>QA 12/10/2026: No se realizaron despliegues ni cambios de ramas/remotos.</t>
+        </is>
+      </c>
+      <c r="M21" s="132" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N21" s="44" t="inlineStr">
+        <is>
+          <t>Codex (QA manual)</t>
+        </is>
+      </c>
+      <c r="O21" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P21" s="44" t="inlineStr">
+        <is>
+          <t>8ef994a</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="68" customHeight="1">
       <c r="A22" s="51" t="inlineStr">

</xml_diff>

<commit_message>
test: registra cierre de casos QA
</commit_message>
<xml_diff>
--- a/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
+++ b/docs/qa/Casos de prueba - Zunino Remates Web.xlsx
@@ -9964,19 +9964,38 @@
       </c>
       <c r="J10" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K10" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K10" s="50" t="inlineStr">
+        <is>
+          <t>Dos remates Mobiliario y antigüedades se publicaron con rutas distintas; el segundo obtuvo mobiliario-y-antiguedades-2 y su detalle público cargó.</t>
+        </is>
+      </c>
       <c r="L10" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): El segundo remate recibió automáticamente el sufijo -2 y el slug no fue editable. Se evitó la colisión antes de publicar.</t>
-        </is>
-      </c>
-      <c r="M10" s="50" t="str"/>
-      <c r="N10" s="50" t="str"/>
-      <c r="O10" s="50" t="str"/>
-      <c r="P10" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): El segundo remate recibió automáticamente el sufijo -2 y el slug no fue editable. Se evitó la colisión antes de publicar.
+Ejecución 2026-10-13: Colisión evitada con sufijo -2; ambos fixtures temporales se eliminaron.</t>
+        </is>
+      </c>
+      <c r="M10" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N10" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O10" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P10" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="68" customHeight="1">
       <c r="A11" s="52" t="inlineStr">
@@ -10112,19 +10131,38 @@
       </c>
       <c r="J12" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K12" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K12" s="50" t="inlineStr">
+        <is>
+          <t>El fixture QA publicado pasó a Finalizado; desapareció de la home y su URL mostró “Remate no encontrado”.</t>
+        </is>
+      </c>
       <c r="L12" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): El remate quedó Finalizado, desapareció de la home y su URL dejó de mostrar el detalle.</t>
-        </is>
-      </c>
-      <c r="M12" s="50" t="str"/>
-      <c r="N12" s="50" t="str"/>
-      <c r="O12" s="50" t="str"/>
-      <c r="P12" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): El remate quedó Finalizado, desapareció de la home y su URL dejó de mostrar el detalle.
+Ejecución 2026-10-13: Validado con fixture temporal QA ESTADOS 2026 y eliminado al finalizar.</t>
+        </is>
+      </c>
+      <c r="M12" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N12" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O12" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P12" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="68" customHeight="1">
       <c r="A13" s="52" t="inlineStr">
@@ -10258,19 +10296,38 @@
       </c>
       <c r="J14" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K14" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K14" s="50" t="inlineStr">
+        <is>
+          <t>El borrador QA-BORRAR - REM-014 se eliminó tras confirmar y no figuró en el listado actualizado.</t>
+        </is>
+      </c>
       <c r="L14" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Al confirmar, el borrador desapareció y no volvió después de recargar.</t>
-        </is>
-      </c>
-      <c r="M14" s="50" t="str"/>
-      <c r="N14" s="50" t="str"/>
-      <c r="O14" s="50" t="str"/>
-      <c r="P14" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Al confirmar, el borrador desapareció y no volvió después de recargar.
+Ejecución 2026-10-13: Validado y limpiado el fixture temporal.</t>
+        </is>
+      </c>
+      <c r="M14" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N14" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O14" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P14" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="68" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
@@ -10323,19 +10380,38 @@
       </c>
       <c r="J15" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K15" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K15" s="44" t="inlineStr">
+        <is>
+          <t>El borrador QA-BORRAR - REM-014 con lugar Sala QA se visualizó desde una segunda pestaña autenticada tras guardarlo.</t>
+        </is>
+      </c>
       <c r="L15" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): El borrador y el lugar guardado permanecieron después de recargar.</t>
-        </is>
-      </c>
-      <c r="M15" s="44" t="str"/>
-      <c r="N15" s="44" t="str"/>
-      <c r="O15" s="44" t="str"/>
-      <c r="P15" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): El borrador y el lugar guardado permanecieron después de recargar.
+Ejecución 2026-10-13: Persistencia comprobada en segunda pestaña; fixture eliminado luego.</t>
+        </is>
+      </c>
+      <c r="M15" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N15" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O15" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P15" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="68" customHeight="1">
       <c r="A16" s="51" t="inlineStr">
@@ -10800,19 +10876,38 @@
       </c>
       <c r="J21" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K21" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K21" s="44" t="inlineStr">
+        <is>
+          <t>Dos remates con el título Remate especial se publicaron con rutas distintas; el segundo recibió remate-especial-2 y su detalle cargó correctamente.</t>
+        </is>
+      </c>
       <c r="L21" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): El segundo título igual recibió un slug terminado en -2 y ambos remates pudieron publicarse.</t>
-        </is>
-      </c>
-      <c r="M21" s="44" t="str"/>
-      <c r="N21" s="44" t="str"/>
-      <c r="O21" s="44" t="str"/>
-      <c r="P21" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): El segundo título igual recibió un slug terminado en -2 y ambos remates pudieron publicarse.
+Ejecución 2026-10-13: Validado con dos fixtures QA; ambos eliminados al finalizar.</t>
+        </is>
+      </c>
+      <c r="M21" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N21" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O21" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P21" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="68" customHeight="1">
       <c r="A22" s="51" t="inlineStr">
@@ -11120,19 +11215,38 @@
       </c>
       <c r="J25" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K25" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K25" s="44" t="inlineStr">
+        <is>
+          <t>El fixture QA CANCELAR 2026 quedó Cancelado; la URL pública devolvió “Remate no encontrado”.</t>
+        </is>
+      </c>
       <c r="L25" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): Al confirmar, quedó Cancelado, desapareció de la home y su URL dejó de mostrar el detalle.</t>
-        </is>
-      </c>
-      <c r="M25" s="44" t="str"/>
-      <c r="N25" s="44" t="str"/>
-      <c r="O25" s="44" t="str"/>
-      <c r="P25" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): Al confirmar, quedó Cancelado, desapareció de la home y su URL dejó de mostrar el detalle.
+Ejecución 2026-10-13: Validado con fixture temporal y eliminado al finalizar.</t>
+        </is>
+      </c>
+      <c r="M25" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N25" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O25" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P25" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="68" customHeight="1">
       <c r="A26" s="51" t="inlineStr">
@@ -11269,19 +11383,38 @@
       </c>
       <c r="J27" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K27" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K27" s="44" t="inlineStr">
+        <is>
+          <t>El título cambió de Remate rural de agosto a Remate rural de setiembre; el slug cambió de remate-rural-de-agosto a remate-rural-de-setiembre y pudo enviarse a revisión.</t>
+        </is>
+      </c>
       <c r="L27" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Aprobado): El slug acompañó el cambio de título en Borrador y En revisión.</t>
-        </is>
-      </c>
-      <c r="M27" s="44" t="str"/>
-      <c r="N27" s="44" t="str"/>
-      <c r="O27" s="44" t="str"/>
-      <c r="P27" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Aprobado): El slug acompañó el cambio de título en Borrador y En revisión.
+Ejecución 2026-10-13: Validado y limpiado el fixture temporal.</t>
+        </is>
+      </c>
+      <c r="M27" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N27" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O27" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P27" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="68" customHeight="1">
       <c r="A28" s="51" t="inlineStr">
@@ -11416,19 +11549,38 @@
       </c>
       <c r="J29" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K29" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K29" s="44" t="inlineStr">
+        <is>
+          <t>En dos pestañas, A guardó Sala A guardada y B recibió conflicto al guardar una descripción obsoleta; los cambios de A se conservaron.</t>
+        </is>
+      </c>
       <c r="L29" s="44" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Falló): La segunda pestaña guardó sin mostrar conflicto y sobrescribió el cambio de lugar de la primera. Después de recargar quedó la descripción de la pestaña B y se perdió el lugar guardado desde A.</t>
-        </is>
-      </c>
-      <c r="M29" s="44" t="str"/>
-      <c r="N29" s="44" t="str"/>
-      <c r="O29" s="44" t="str"/>
-      <c r="P29" s="44" t="str"/>
+          <t>Histórico de la versión anterior (Falló): La segunda pestaña guardó sin mostrar conflicto y sobrescribió el cambio de lugar de la primera. Después de recargar quedó la descripción de la pestaña B y se perdió el lugar guardado desde A.
+Ejecución 2026-10-13: Corregido en el Preview: B mostró aviso de modificación concurrente y no guardó la versión obsoleta. Fixture eliminado luego.</t>
+        </is>
+      </c>
+      <c r="M29" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N29" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O29" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P29" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="68" customHeight="1">
       <c r="A30" s="51" t="inlineStr">
@@ -11479,19 +11631,39 @@
       </c>
       <c r="J30" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K30" s="50" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K30" s="50" t="inlineStr">
+        <is>
+          <t>En dos pestañas, la acción Ocultar de la versión desactualizada se aplicó; el guardado paralelo mostró conflicto. El fixture se restauró y se eliminó.</t>
+        </is>
+      </c>
       <c r="L30" s="50" t="inlineStr">
         <is>
-          <t>Histórico de la versión anterior (Falló): La pestaña desactualizada ocultó el remate sin aviso y perdió el cambio guardado desde la otra pestaña. No se mostró conflicto de versión; el estado final fue Oculto.</t>
-        </is>
-      </c>
-      <c r="M30" s="50" t="str"/>
-      <c r="N30" s="50" t="str"/>
-      <c r="O30" s="50" t="str"/>
-      <c r="P30" s="50" t="str"/>
+          <t>Histórico de la versión anterior (Falló): La pestaña desactualizada ocultó el remate sin aviso y perdió el cambio guardado desde la otra pestaña. No se mostró conflicto de versión; el estado final fue Oculto.
+Histórico de la versión anterior (Falló): La pestaña desactualizada ocultó el remate sin aviso y perdió el cambio guardado desde la otra pestaña. No se mostró conflicto de versión; el estado final fue Oculto.
+Ejecución 2026-10-13: Reproducido. La mutación de estado no rechazó la versión desactualizada; el control de concurrencia se mostró en el guardado paralelo, no al ocultar.</t>
+        </is>
+      </c>
+      <c r="M30" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N30" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O30" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P30" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="68" customHeight="1">
       <c r="A31" s="52" t="inlineStr">
@@ -11873,15 +12045,37 @@
       </c>
       <c r="J35" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K35" s="44" t="str"/>
-      <c r="L35" s="44" t="str"/>
-      <c r="M35" s="44" t="str"/>
-      <c r="N35" s="44" t="str"/>
-      <c r="O35" s="44" t="str"/>
-      <c r="P35" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K35" s="44" t="inlineStr">
+        <is>
+          <t>No fue posible simular Offline de manera controlada en el Preview protegido sin alterar la conectividad compartida del entorno.</t>
+        </is>
+      </c>
+      <c r="L35" s="44" t="inlineStr">
+        <is>
+          <t>Requiere emulación de red aislada (DevTools/entorno local) para verificar que no aparezca éxito falso durante un guardado. No se modificaron datos para este caso.</t>
+        </is>
+      </c>
+      <c r="M35" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N35" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O35" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P35" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="68" customHeight="1">
       <c r="A36" s="51" t="inlineStr">
@@ -12176,15 +12370,37 @@
       </c>
       <c r="J39" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K39" s="44" t="str"/>
-      <c r="L39" s="44" t="str"/>
-      <c r="M39" s="44" t="str"/>
-      <c r="N39" s="44" t="str"/>
-      <c r="O39" s="44" t="str"/>
-      <c r="P39" s="44" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K39" s="44" t="inlineStr">
+        <is>
+          <t>Tras guardar una edición en A, B intentó eliminar una versión obsoleta y recibió “El remate cambió. Recargá el listado antes de eliminarlo.”; el remate se conservó.</t>
+        </is>
+      </c>
+      <c r="L39" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Conflicto de borrado rechazado correctamente; fixture eliminado luego con versión vigente.</t>
+        </is>
+      </c>
+      <c r="M39" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N39" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O39" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P39" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="68" customHeight="1">
       <c r="A40" s="51" t="inlineStr">
@@ -20199,15 +20415,37 @@
       </c>
       <c r="J3" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K3" s="44" t="str"/>
-      <c r="L3" s="44" t="str"/>
-      <c r="M3" s="44" t="str"/>
-      <c r="N3" s="44" t="str"/>
-      <c r="O3" s="44" t="str"/>
-      <c r="P3" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K3" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere una instancia o despliegue aislado con la base inaccesible. No se pausó el proyecto Supabase compartido.</t>
+        </is>
+      </c>
+      <c r="L3" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere una instancia o despliegue aislado con la base inaccesible. No se pausó el proyecto Supabase compartido.</t>
+        </is>
+      </c>
+      <c r="M3" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N3" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O3" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P3" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="68" customHeight="1">
       <c r="A4" s="51" t="inlineStr">
@@ -20420,15 +20658,37 @@
       </c>
       <c r="J6" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K6" s="50" t="str"/>
-      <c r="L6" s="50" t="str"/>
-      <c r="M6" s="50" t="str"/>
-      <c r="N6" s="50" t="str"/>
-      <c r="O6" s="50" t="str"/>
-      <c r="P6" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K6" s="50" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere solicitudes HTTP manuales POST/PUT contra endpoints públicos. El Preview está protegido por Vercel y no expone un canal HTTP autenticado para inspección manual.</t>
+        </is>
+      </c>
+      <c r="L6" s="50" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere solicitudes HTTP manuales POST/PUT contra endpoints públicos. El Preview está protegido por Vercel y no expone un canal HTTP autenticado para inspección manual.</t>
+        </is>
+      </c>
+      <c r="M6" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N6" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O6" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P6" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="68" customHeight="1">
       <c r="A7" s="52" t="inlineStr">
@@ -20479,15 +20739,37 @@
       </c>
       <c r="J7" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K7" s="44" t="str"/>
-      <c r="L7" s="44" t="str"/>
-      <c r="M7" s="44" t="str"/>
-      <c r="N7" s="44" t="str"/>
-      <c r="O7" s="44" t="str"/>
-      <c r="P7" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K7" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere una sesión sin cookie y acceso directo a endpoints privados. El navegador disponible comparte la sesión autenticada y el acceso HTTP directo está cubierto por Vercel Authentication.</t>
+        </is>
+      </c>
+      <c r="L7" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere una sesión sin cookie y acceso directo a endpoints privados. El navegador disponible comparte la sesión autenticada y el acceso HTTP directo está cubierto por Vercel Authentication.</t>
+        </is>
+      </c>
+      <c r="M7" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N7" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O7" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P7" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="68" customHeight="1">
       <c r="A8" s="51" t="inlineStr">
@@ -20538,15 +20820,37 @@
       </c>
       <c r="J8" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K8" s="50" t="str"/>
-      <c r="L8" s="50" t="str"/>
-      <c r="M8" s="50" t="str"/>
-      <c r="N8" s="50" t="str"/>
-      <c r="O8" s="50" t="str"/>
-      <c r="P8" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K8" s="50" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere variar Origin y CSRF en solicitudes autenticadas. El Preview protegido no permite inyectar cabeceras personalizadas desde el flujo manual disponible.</t>
+        </is>
+      </c>
+      <c r="L8" s="50" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere variar Origin y CSRF en solicitudes autenticadas. El Preview protegido no permite inyectar cabeceras personalizadas desde el flujo manual disponible.</t>
+        </is>
+      </c>
+      <c r="M8" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N8" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O8" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P8" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="68" customHeight="1">
       <c r="A9" s="52" t="inlineStr">
@@ -20597,15 +20901,37 @@
       </c>
       <c r="J9" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K9" s="44" t="str"/>
-      <c r="L9" s="44" t="str"/>
-      <c r="M9" s="44" t="str"/>
-      <c r="N9" s="44" t="str"/>
-      <c r="O9" s="44" t="str"/>
-      <c r="P9" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K9" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere inspeccionar cabeceras HTTP privadas en una respuesta directa. Vercel Authentication bloquea las solicitudes no interactivas al Preview.</t>
+        </is>
+      </c>
+      <c r="L9" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere inspeccionar cabeceras HTTP privadas en una respuesta directa. Vercel Authentication bloquea las solicitudes no interactivas al Preview.</t>
+        </is>
+      </c>
+      <c r="M9" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N9" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O9" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P9" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="68" customHeight="1">
       <c r="A10" s="51" t="inlineStr">
@@ -20819,15 +21145,37 @@
       </c>
       <c r="J12" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K12" s="50" t="str"/>
-      <c r="L12" s="50" t="str"/>
-      <c r="M12" s="50" t="str"/>
-      <c r="N12" s="50" t="str"/>
-      <c r="O12" s="50" t="str"/>
-      <c r="P12" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K12" s="50" t="inlineStr">
+        <is>
+          <t>La segunda escritura con versión obsoleta fue rechazada desde la UI con aviso de modificación concurrente; se preservó la versión guardada por A.</t>
+        </is>
+      </c>
+      <c r="L12" s="50" t="inlineStr">
+        <is>
+          <t>Ejecución manual equivalente mediante dos pestañas autenticadas. La UI no expone el código HTTP, pero el comportamiento observable corresponde al rechazo de conflicto requerido. Fixture QA eliminado luego.</t>
+        </is>
+      </c>
+      <c r="M12" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N12" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O12" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P12" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="68" customHeight="1">
       <c r="A13" s="52" t="inlineStr">
@@ -20878,15 +21226,37 @@
       </c>
       <c r="J13" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K13" s="44" t="str"/>
-      <c r="L13" s="44" t="str"/>
-      <c r="M13" s="44" t="str"/>
-      <c r="N13" s="44" t="str"/>
-      <c r="O13" s="44" t="str"/>
-      <c r="P13" s="44" t="str"/>
+          <t>Falló</t>
+        </is>
+      </c>
+      <c r="K13" s="44" t="inlineStr">
+        <is>
+          <t>El borrado obsoleto fue rechazado, pero la ocultación desde una versión desactualizada se aplicó en la prueba de carrera.</t>
+        </is>
+      </c>
+      <c r="L13" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución manual equivalente: DELETE stale protegido; hide stale no protegido de forma consistente. Fixture restaurado y eliminado.</t>
+        </is>
+      </c>
+      <c r="M13" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N13" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O13" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P13" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="68" customHeight="1">
       <c r="A14" s="51" t="inlineStr">
@@ -20936,15 +21306,37 @@
       </c>
       <c r="J14" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K14" s="50" t="str"/>
-      <c r="L14" s="50" t="str"/>
-      <c r="M14" s="50" t="str"/>
-      <c r="N14" s="50" t="str"/>
-      <c r="O14" s="50" t="str"/>
-      <c r="P14" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K14" s="50" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere perfiles activos de editor y administrador en sesiones separadas. No se dispone de una vía segura en este Preview para provisionar y asignar perfiles de rol sin alterar configuración compartida.</t>
+        </is>
+      </c>
+      <c r="L14" s="50" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere perfiles activos de editor y administrador en sesiones separadas. No se dispone de una vía segura en este Preview para provisionar y asignar perfiles de rol sin alterar configuración compartida.</t>
+        </is>
+      </c>
+      <c r="M14" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N14" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O14" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P14" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="68" customHeight="1">
       <c r="A15" s="52" t="inlineStr">
@@ -20995,15 +21387,37 @@
       </c>
       <c r="J15" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K15" s="44" t="str"/>
-      <c r="L15" s="44" t="str"/>
-      <c r="M15" s="44" t="str"/>
-      <c r="N15" s="44" t="str"/>
-      <c r="O15" s="44" t="str"/>
-      <c r="P15" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K15" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere Storage configurado, una foto de remate publicada y verificación de URL firmada frente a ruta directa. No hubo un fixture de archivo/Storage aislado disponible.</t>
+        </is>
+      </c>
+      <c r="L15" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere Storage configurado, una foto de remate publicada y verificación de URL firmada frente a ruta directa. No hubo un fixture de archivo/Storage aislado disponible.</t>
+        </is>
+      </c>
+      <c r="M15" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N15" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O15" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P15" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="68" customHeight="1">
       <c r="A16" s="51" t="inlineStr">
@@ -21054,15 +21468,37 @@
       </c>
       <c r="J16" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K16" s="50" t="str"/>
-      <c r="L16" s="50" t="str"/>
-      <c r="M16" s="50" t="str"/>
-      <c r="N16" s="50" t="str"/>
-      <c r="O16" s="50" t="str"/>
-      <c r="P16" s="50" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K16" s="50" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere archivos controlados con tamaños, MIME y firmas específicas, además de observar la limpieza de cargas parciales. No se ejecutó contra Storage compartido sin sandbox de archivos.</t>
+        </is>
+      </c>
+      <c r="L16" s="50" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere archivos controlados con tamaños, MIME y firmas específicas, además de observar la limpieza de cargas parciales. No se ejecutó contra Storage compartido sin sandbox de archivos.</t>
+        </is>
+      </c>
+      <c r="M16" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N16" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O16" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P16" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="68" customHeight="1">
       <c r="A17" s="52" t="inlineStr">
@@ -21114,15 +21550,37 @@
       </c>
       <c r="J17" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K17" s="44" t="str"/>
-      <c r="L17" s="44" t="str"/>
-      <c r="M17" s="44" t="str"/>
-      <c r="N17" s="44" t="str"/>
-      <c r="O17" s="44" t="str"/>
-      <c r="P17" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K17" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere forzar un fallo entre carga y guardado y comprobar el borrado de huérfanos. No se puede inducir esa falla de manera aislada desde el Preview protegido.</t>
+        </is>
+      </c>
+      <c r="L17" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere forzar un fallo entre carga y guardado y comprobar el borrado de huérfanos. No se puede inducir esa falla de manera aislada desde el Preview protegido.</t>
+        </is>
+      </c>
+      <c r="M17" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N17" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O17" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P17" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="68" customHeight="1">
       <c r="A18" s="51" t="inlineStr">
@@ -21498,15 +21956,37 @@
       </c>
       <c r="J22" s="50" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K22" s="50" t="str"/>
-      <c r="L22" s="50" t="str"/>
-      <c r="M22" s="50" t="str"/>
-      <c r="N22" s="50" t="str"/>
-      <c r="O22" s="50" t="str"/>
-      <c r="P22" s="50" t="str"/>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="K22" s="50" t="inlineStr">
+        <is>
+          <t>La auditoría registró INSERT, UPDATE y DELETE de los fixtures QA de remates, con entidad, acción, registro y fecha; no se observaron datos sensibles de consultas.</t>
+        </is>
+      </c>
+      <c r="L22" s="50" t="inlineStr">
+        <is>
+          <t>Verificado mediante consulta de solo lectura a public.audit_log luego de las operaciones QA. Los fixtures temporales fueron eliminados.</t>
+        </is>
+      </c>
+      <c r="M22" s="117" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N22" s="50" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O22" s="50" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P22" s="50" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="68" customHeight="1">
       <c r="A23" s="52" t="inlineStr">
@@ -21557,15 +22037,37 @@
       </c>
       <c r="J23" s="44" t="inlineStr">
         <is>
-          <t>No ejecutado</t>
-        </is>
-      </c>
-      <c r="K23" s="44" t="str"/>
-      <c r="L23" s="44" t="str"/>
-      <c r="M23" s="44" t="str"/>
-      <c r="N23" s="44" t="str"/>
-      <c r="O23" s="44" t="str"/>
-      <c r="P23" s="44" t="str"/>
+          <t>Bloqueado</t>
+        </is>
+      </c>
+      <c r="K23" s="44" t="inlineStr">
+        <is>
+          <t>No ejecutado: Requiere una cuenta Auth sin perfil activo y una sesión separada. No se provisionó esa combinación en el entorno compartido durante esta ejecución.</t>
+        </is>
+      </c>
+      <c r="L23" s="44" t="inlineStr">
+        <is>
+          <t>Ejecución 2026-10-13: Requiere una cuenta Auth sin perfil activo y una sesión separada. No se provisionó esa combinación en el entorno compartido durante esta ejecución.</t>
+        </is>
+      </c>
+      <c r="M23" s="116" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N23" s="44" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="O23" s="44" t="inlineStr">
+        <is>
+          <t>Vercel Preview protegido (Edge)</t>
+        </is>
+      </c>
+      <c r="P23" s="44" t="inlineStr">
+        <is>
+          <t>c908923 (rama codex/nuevo-diseno-home)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>